<commit_message>
cf optimization, testing, idk how this code works but it does...mostly
</commit_message>
<xml_diff>
--- a/data/matching_tabelle.xlsx
+++ b/data/matching_tabelle.xlsx
@@ -425,29 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D137"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name_dem_24</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name_dem_24</t>
+          <t>Name_fm</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Name_fm</t>
+          <t>Name_dem_23</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Name_dem_23</t>
+          <t>Name_sat_23</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Name_sat_24</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>aokbadenwürttemberg</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -461,13 +473,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>aokbadenwürttemberg</t>
+          <t>badenwürtt.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>badenwürtt.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>aokbayern</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -481,13 +500,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>aokbayern</t>
+          <t>bayern</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bayern</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>aokhessen</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -501,13 +527,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>aokhessen</t>
+          <t>hessen</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>hessen</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>aokniedersachsen</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -521,13 +554,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>aokniedersachsen</t>
+          <t>niedersachsen</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>niedersachsen</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>aoknordost</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -541,13 +581,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>aoknordost</t>
+          <t>nordost</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nordost</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>5</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>aoknordwest</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -561,13 +608,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>aoknordwest</t>
+          <t>nordwest</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nordwest</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>6</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aokplus</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -581,13 +635,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>aokplus</t>
+          <t>plus</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>plus</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>7</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>aokrheinland/hamburg</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -601,13 +662,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>aokrheinland/hamburg</t>
+          <t>rheinl./hamburg</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>rheinl./hamburg</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>8</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>aokrheinlandpfalz/saarland</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -621,13 +689,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>aokrheinlandpfalz/saarland</t>
+          <t>rheinl.pfalz/saarland</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>rheinl.pfalz/saarland</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>9</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>aoksachsenanhalt</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -641,13 +716,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>aoksachsenanhalt</t>
+          <t>sachs.anhalt</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sachs.anhalt</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>10</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>audibkk</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -664,10 +746,17 @@
           <t>audibkk</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>audibkk</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>11</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>bahnbkk</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -684,10 +773,17 @@
           <t>bahnbkk</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>bahnbkk</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>12</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>barmer</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -704,10 +800,17 @@
           <t>barmer</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>barmer</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>13</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>bigdirektgesund</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -724,10 +827,17 @@
           <t>bigdirektgesund</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>bigdirektgesund</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>14</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>bkk24</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -744,10 +854,17 @@
           <t>bkk24</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>bkk24</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>bkkdeutschebankag</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -761,13 +878,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>bkkdeutschebankag</t>
+          <t>bkkdeutschebank</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>bkkdeutschebank</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>16</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>bkkeuregio</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -784,10 +908,17 @@
           <t>bkkeuregio</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>bkkeuregio</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>17</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>bkkfabercastell&amp;partner</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -801,13 +932,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>bkkfabercastell&amp;partner</t>
+          <t>bkkfabercastell</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>bkkfabercastell</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>bkkfirmus</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -824,10 +962,17 @@
           <t>bkkfirmus</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>bkkfirmus</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>bkkgildemeisterseidensticker</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -841,13 +986,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>bkkgildemeisterseidensticker</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>bkkgs</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>bkklinde</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -864,10 +1016,17 @@
           <t>bkklinde</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>bkklinde</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>bkkpfalz</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -884,10 +1043,17 @@
           <t>bkkpfalz</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>bkkpfalz</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>bkkprovita</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -904,10 +1070,17 @@
           <t>bkkprovita</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>bkkprovita</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>bkkscheufelen</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -924,10 +1097,17 @@
           <t>bkkscheufelen</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>bkkscheufelen</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>bmwbkk</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -944,10 +1124,17 @@
           <t>bmwbkk</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>bmwbkk</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>boschbkk</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -964,10 +1151,17 @@
           <t>boschbkk</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>boschbkk</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>26</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>dakgesundheit</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -984,10 +1178,17 @@
           <t>dakgesundheit</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>dakgesundheit</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>27</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>debekabkk</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1004,10 +1205,17 @@
           <t>debekabkk</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>debekabkk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>28</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>heimatkrankenkasse</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1021,13 +1229,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>heimatkrankenkasse</t>
+          <t>heimatkk</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>heimatkk</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>29</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>hek</t>
+        </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1044,30 +1259,44 @@
           <t>hek</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>hek</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
-        <v>30</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>hkkkrankenkasse</t>
+        </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>hkkkrankenkasse</t>
+          <t>hkk</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>hkk</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>sonstigegkv</t>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>hkk</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>31</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ikkbrandenburgundberlin</t>
+        </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1081,13 +1310,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ikkbrandenburgundberlin</t>
+          <t>ikkbrandenburg/berlin</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ikkbrandenburg/berlin</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>32</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ikkclassic</t>
+        </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1101,13 +1337,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ikkclassic</t>
+          <t>ikkquadclassic</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ikkquadclassic</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>33</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ikkdieinnovationskasse</t>
+        </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1124,10 +1367,17 @@
           <t>ikkdieinnovationskasse</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ikkdieinnovationskasse</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>34</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ikkgesundplus</t>
+        </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1144,10 +1394,17 @@
           <t>ikkgesundplus</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ikkgesundplus</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>35</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ikksüdwest</t>
+        </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1164,30 +1421,44 @@
           <t>ikksüdwest</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ikksüdwest</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>36</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>kkh</t>
+        </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>kaufmännischekrankenkasse(kkh)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
           <t>kkh</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>kaufmännischekrankenkasse(kkh)</t>
-        </is>
-      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>kkh</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>kkh</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>37</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>knappschaft</t>
+        </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1204,10 +1475,17 @@
           <t>knappschaft</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>knappschaft</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>38</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mercedesbenzbkk</t>
+        </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1224,14 +1502,21 @@
           <t>mercedesbenzbkk</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>mercedesbenzbkk</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mhpluskrankenkasse</t>
+        </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>mhpluskrankenkasse</t>
+          <t>mhplusbkk</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1244,50 +1529,71 @@
           <t>mhplusbkk</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>mhplusbkk</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mkkmeinekrankenkasse</t>
+        </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>mkkmeinekrankenkasse</t>
+          <t>bkkmkkmeinekrankenkasse</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>bkkmkkmeinekrankenkasse</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mobilkrankenkasse</t>
+        </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>betriebskrankenkassemobil</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
           <t>mobilkrankenkasse</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>betriebskrankenkassemobil</t>
-        </is>
-      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>mobilkrankenkasse</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>mobilkrankenkasse</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>novitasbkk</t>
+        </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1304,10 +1610,17 @@
           <t>novitasbkk</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>novitasbkk</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>pronovabkk</t>
+        </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1324,30 +1637,44 @@
           <t>pronovabkk</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>pronovabkk</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>r+vbkk</t>
+        </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>r+vbetriebskrankenkasse</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
           <t>r+vbkk</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>r+vbetriebskrankenkasse</t>
-        </is>
-      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>r+vbkk</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>r+vbkk</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>salusbkk</t>
+        </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1364,10 +1691,17 @@
           <t>salusbkk</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>salusbkk</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>sbk</t>
+        </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1384,50 +1718,71 @@
           <t>sbk</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>sbk</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>securvita</t>
+        </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>securvitabkk</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
           <t>securvita</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>securvitabkk</t>
-        </is>
-      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>securvita</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>securvita</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>technikerkrankenkasse(tk)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
           <t>tk</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>technikerkrankenkasse(tk)</t>
-        </is>
-      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>tk</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>tk</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>viactivkrankenkasse</t>
+        </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1441,13 +1796,20 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>viactivkrankenkasse</t>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>viactivkk</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>vividabkk</t>
+        </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1464,19 +1826,26 @@
           <t>vividabkk</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>vividabkk</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>actimondakrankenkasse</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>actimondakrankenkasse</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1484,1199 +1853,1619 @@
           <t>sonstigegkv</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>aok</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
           <t>aok</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>sonstigegkv</t>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>aok</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>aokbremen/bremerhaven</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>aokbremen/bremerhaven</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>aokgesamt</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>aokgesamt</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>54</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>atlasbkkahlmann</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>atlasbkkahlmann</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>55</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bertelsmannbkk</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>bertelsmannbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>56</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkachenbachbuschhütten</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>bkkachenbachbuschhütten</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>57</v>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkadvita</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>bkkadvita</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>58</v>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkaesculap</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>bkkaesculap</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>59</v>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkakzonobelbayern</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>bkkakzonobelbayern</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>60</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkb.braunaesculap</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>bkkb.braunaesculap</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>61</v>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkbasell</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>bkkbasell</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>62</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkbeiersdorfag</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>bkkbeiersdorfag</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>63</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkbjb</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>bkkbjb</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>64</v>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkbpwbergischeachsen</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>bkkbpwbergischeachsen</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>65</v>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkbraungillette</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>bkkbraungillette</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>66</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkdemagkraussmaffei</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>bkkdemagkraussmaffei</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>67</v>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkdiakonie</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>bkkdiakonie</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>68</v>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkdürkoppadler</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>bkkdürkoppadler</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
-        <v>69</v>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkessanelle</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>bkkessanelle</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
-        <v>70</v>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkevm</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>bkkevm</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
-        <v>71</v>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkewe</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>bkkewe</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
-        <v>72</v>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkexklusiv</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>bkkexklusiv</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
-        <v>73</v>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkfamily(ehem.bkkihv)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>bkkfamily(ehem.bkkihv)</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
-        <v>74</v>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkfreudenberg</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>bkkfreudenberg</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
-        <v>75</v>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgrillowerke</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>bkkgrillowerke</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
-        <v>76</v>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgrozbeckert</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>bkkgrozbeckert</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
-        <v>77</v>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkhenschelplus</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>bkkhenschelplus</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
-        <v>78</v>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkherfordmindenravensberg</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>bkkherfordmindenravensberg</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
-        <v>79</v>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkherkules</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>bkkherkules</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
-        <v>80</v>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkhmr</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>bkkhmr</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
-        <v>81</v>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkkarlmayer</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>bkkkarlmayer</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
-        <v>82</v>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkkassana</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>bkkkassana</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
-        <v>83</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmahle</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>bkkmahle</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
-        <v>84</v>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmedicus</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>bkkmedicus</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
-        <v>85</v>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmelittahmr</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>bkkmelittahmr</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
-        <v>86</v>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmem</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>bkkmem</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
-        <v>87</v>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmerck</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>bkkmerck</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
-        <v>88</v>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmiele</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>bkkmiele</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
-        <v>89</v>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkmtu</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>bkkmtu</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
-        <v>90</v>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkpfaff</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>bkkpfaff</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
-        <v>91</v>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkpublic</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>bkkpublic</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
-        <v>92</v>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkpwc</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>bkkpwc</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
-        <v>93</v>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkrieker.ricosta.weisser</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>bkkrieker.ricosta.weisser</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
-        <v>94</v>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkrwe</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>bkkrwe</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
-        <v>95</v>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkksalzgitter</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>bkksalzgitter</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
-        <v>96</v>
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkksbh</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>bkksbh</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
-        <v>97</v>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkschleswigholstein</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>bkkschleswigholstein</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
-        <v>98</v>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkstadtaugsburg</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>bkkstadtaugsburg</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
-        <v>99</v>
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkktechnoform</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>bkktechnoform</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
-        <v>100</v>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkktextilgruppehof</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>bkktextilgruppehof</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
-        <v>101</v>
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkvdn</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>bkkvdn</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
-        <v>102</v>
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkverbundplus</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
           <t>bkkverbundplus</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>sonstigegkv</t>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>bkkverbundplus</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
-        <v>103</v>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkvictoriad.a.s</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>bkkvictoriad.a.s</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
-        <v>104</v>
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkvital</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>bkkvital</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
-        <v>105</v>
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkvoralbheller*index*leuze</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>bkkvoralbheller*index*leuze</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
-        <v>106</v>
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkwerrameissner</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>bkkwerrameissner</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
-        <v>107</v>
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkwirtschaftundfinanzen</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>bkkwirtschaftundfinanzen</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
-        <v>108</v>
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkwürth</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>bkkwürth</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
-        <v>109</v>
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkzf&amp;partner</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>bkkzf&amp;partner</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
-        <v>110</v>
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>brandenburgischebkk</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>brandenburgischebkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
-        <v>111</v>
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>continentalebetriebskrankenkasse</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>continentalebetriebskrankenkasse</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2684,139 +3473,188 @@
           <t>sonstigegkv</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
-        <v>112</v>
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>deutschebkk</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>deutschebkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
-        <v>113</v>
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>diebergischekrankenkasse</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>diebergischekrankenkasse</t>
+          <t>bergischekrankenkasse</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>bergischekrankenkasse</t>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
-        <v>114</v>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>e.onbkk</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>e.onbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
-        <v>115</v>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>energiebkk</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>energiebkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
-        <v>116</v>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>essobkk</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>essobkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
-        <v>117</v>
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>eybkk</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>eybkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
-        <v>118</v>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>gkv</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>gkv</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -2824,179 +3662,242 @@
           <t>sonstigegkv</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
-        <v>119</v>
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>heagbkk</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>heagbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
-        <v>120</v>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>ikk</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
           <t>ikk</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>sonstigegkv</t>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ikk</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
-        <v>121</v>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>koenig&amp;bauerbkk</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>koenig&amp;bauerbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
-        <v>122</v>
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>kronesbkk</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>kronesbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
-        <v>123</v>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>metzingerbkk</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>metzingerbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
-        <v>124</v>
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>shellbkklife</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>shellbkklife</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
-        <v>125</v>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>siemagbkk</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>siemagbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
-        <v>126</v>
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>skdbkk</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>skdbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
-        <v>127</v>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>svlfg</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>svlfg</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -3004,39 +3905,53 @@
           <t>sonstigegkv</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
-        <v>128</v>
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>südzuckerbkk</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>südzuckerbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
-        <v>129</v>
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>tbkthüringerbetriebskrankenkasse</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>tbkthüringerbetriebskrankenkasse</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3044,59 +3959,80 @@
           <t>sonstigegkv</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
-        <v>130</v>
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>tuibkk</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>tuibkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
-        <v>131</v>
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>vaillantbkk</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>vaillantbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
-        <v>132</v>
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>vdek</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>vdek</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -3104,64 +4040,90 @@
           <t>sonstigegkv</t>
         </is>
       </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
-        <v>133</v>
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>vereinigtebkk</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>vereinigtebkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
-        <v>134</v>
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>wielandbkk</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>wielandbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
-        <v>135</v>
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>sonstigegkv</t>
+        </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>wmfbkk</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>wmfbkk</t>
+          <t>sonstigegkv</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>sonstigegkv</t>
+          <t>bkkgesamt</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>bkkgesamt</t>
         </is>
       </c>
     </row>

</xml_diff>